<commit_message>
Data export W37-2026 (2026-09-19T10:07:34Z)
</commit_message>
<xml_diff>
--- a/files/energy_dashboard/energy_dashboard_March_2026.xlsx
+++ b/files/energy_dashboard/energy_dashboard_March_2026.xlsx
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="B29" s="10" t="n">
-        <v>3407</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="30">
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="B30" s="8" t="n">
-        <v>3236</v>
+        <v>4300</v>
       </c>
     </row>
     <row r="31">
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>171</v>
+        <v>90</v>
       </c>
     </row>
     <row r="32">
@@ -1030,7 +1030,7 @@
         </is>
       </c>
       <c r="B37" s="16" t="n">
-        <v>171</v>
+        <v>90</v>
       </c>
     </row>
     <row r="38">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>5%</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1059,7 @@
       </c>
       <c r="C39" s="14" t="inlineStr">
         <is>
-          <t>21%</t>
+          <t>16%</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>23%</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C41" s="14" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>17%</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="C42" s="14" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>9%</t>
         </is>
       </c>
     </row>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C43" s="14" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>4%</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>3%</t>
+          <t>2%</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>171</v>
+        <v>90</v>
       </c>
     </row>
     <row r="22">
@@ -1272,7 +1272,7 @@
         </is>
       </c>
       <c r="C22" s="23" t="n">
-        <v>3236</v>
+        <v>4300</v>
       </c>
     </row>
     <row r="23">
@@ -1282,7 +1282,7 @@
         </is>
       </c>
       <c r="C23" s="20" t="n">
-        <v>3407</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="35">
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="C36" s="22" t="n">
-        <v>171</v>
+        <v>90</v>
       </c>
     </row>
     <row r="37">
@@ -1453,113 +1453,113 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>W10-2026</t>
+          <t>W13-2026</t>
         </is>
       </c>
       <c r="B3" s="14" t="n">
-        <v>16098</v>
+        <v>18160</v>
       </c>
       <c r="C3" s="14" t="n">
-        <v>15007</v>
+        <v>16266</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>457</v>
+        <v>791</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>260</v>
+        <v>379</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>374</v>
+        <v>724</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>16098</v>
+        <v>18160</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>14520</v>
+        <v>34531</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>W11-2026</t>
+          <t>W14-2026</t>
         </is>
       </c>
       <c r="B4" s="14" t="n">
-        <v>15926</v>
+        <v>20846</v>
       </c>
       <c r="C4" s="14" t="n">
-        <v>14499</v>
+        <v>18355</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>607</v>
+        <v>974</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>328</v>
+        <v>470</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>492</v>
+        <v>1047</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>15926</v>
+        <v>20846</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>19931</v>
+        <v>34082</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>W12-2026</t>
+          <t>W15-2026</t>
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>12285</v>
+        <v>14186</v>
       </c>
       <c r="C5" s="14" t="n">
-        <v>11119</v>
+        <v>12699</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>510</v>
+        <v>647</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>266</v>
+        <v>327</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>390</v>
+        <v>513</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>12285</v>
+        <v>14186</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>20358</v>
+        <v>23522</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>W13-2026</t>
+          <t>W16-2026</t>
         </is>
       </c>
       <c r="B6" s="14" t="n">
-        <v>18160</v>
+        <v>13540</v>
       </c>
       <c r="C6" s="14" t="n">
-        <v>16266</v>
+        <v>12034</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>791</v>
+        <v>607</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>379</v>
+        <v>368</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>724</v>
+        <v>531</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>18160</v>
+        <v>13540</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>34531</v>
+        <v>26733</v>
       </c>
     </row>
     <row r="7">
@@ -1569,25 +1569,25 @@
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>62469</v>
+        <v>66732</v>
       </c>
       <c r="C7" s="26" t="n">
-        <v>56891</v>
+        <v>59354</v>
       </c>
       <c r="D7" s="26" t="n">
-        <v>2365</v>
+        <v>3019</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>1233</v>
+        <v>1544</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>1980</v>
+        <v>2815</v>
       </c>
       <c r="G7" s="26" t="n">
-        <v>62469</v>
+        <v>66732</v>
       </c>
       <c r="H7" s="26" t="n">
-        <v>89340</v>
+        <v>118868</v>
       </c>
     </row>
   </sheetData>

</xml_diff>